<commit_message>
RELX: re-run valuation after evidence audit (1,821p SELL)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/RELX/2026-10-14/valuation/dcf.xlsx
+++ b/runs/RELX/2026-10-14/valuation/dcf.xlsx
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.05</v>
+        <v>0.042</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2044.926705519653</v>
+        <v>2102.881781249673</v>
       </c>
     </row>
     <row r="16">
@@ -1392,7 +1392,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.103145</v>
+        <v>0.0953618</v>
       </c>
     </row>
     <row r="18">
@@ -1420,7 +1420,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.09600960394000001</v>
+        <v>0.089224054516</v>
       </c>
     </row>
     <row r="20">
@@ -1434,7 +1434,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>11133.7332424089</v>
+        <v>11302.6880463898</v>
       </c>
     </row>
     <row r="21">
@@ -1462,7 +1462,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>37880.3647832059</v>
+        <v>41593.51174104817</v>
       </c>
     </row>
     <row r="23">
@@ -1476,7 +1476,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>25075.49608778312</v>
+        <v>28313.79494258443</v>
       </c>
     </row>
     <row r="24">
@@ -1490,7 +1490,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>36209.22933019201</v>
+        <v>39616.48298897423</v>
       </c>
     </row>
     <row r="25">
@@ -1518,7 +1518,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>29212.22933019201</v>
+        <v>32619.48298897423</v>
       </c>
     </row>
     <row r="27">
@@ -1532,7 +1532,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>28274.65980173853</v>
+        <v>31759.43622156893</v>
       </c>
     </row>
     <row r="28">
@@ -1546,7 +1546,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>16.21481471214875</v>
+        <v>18.21324738497407</v>
       </c>
     </row>
     <row r="29">
@@ -1560,7 +1560,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1621.481471214875</v>
+        <v>1821.324738497407</v>
       </c>
     </row>
     <row r="30">
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>-0.4148388772</v>
+        <v>-0.3427193293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>